<commit_message>
feat - Stored extra times in separate file.
</commit_message>
<xml_diff>
--- a/extras.xlsx
+++ b/extras.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -58,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -540,19 +536,9 @@
           <t>Filmon</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1490851</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>41810</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Dolphins</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>1.11.50</t>
@@ -599,19 +585,9 @@
           <t>Myronov</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1673595</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>41951</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Dolphins</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>55.09</t>
@@ -658,19 +634,9 @@
           <t>Smith</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1739168</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>41836</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Dolphins</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
         <v>58.25</v>
       </c>
@@ -711,19 +677,9 @@
           <t>Clarke</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1765402</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>42086</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Dolphins</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>54.91</v>
@@ -758,19 +714,9 @@
           <t>Peksa</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1648221</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>41211</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Dolphins</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>1.12.25</t>
@@ -809,19 +755,9 @@
           <t>Bellenger</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1772739</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>41353</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Dolphins</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>1.11.25</t>
@@ -860,19 +796,9 @@
           <t>Obiamiwe</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1595685</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>41570</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Dolphins</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>53.81</v>
       </c>
@@ -915,19 +841,9 @@
           <t>Pitzioris</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1653488</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>41584</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Dolphins</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
         <v>59.38</v>
       </c>
@@ -962,19 +878,9 @@
           <t>Leung</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1684191</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>41946</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Herrings</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>59.91</t>
@@ -1021,19 +927,9 @@
           <t>O'Neill</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1592376</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>41919</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Herrings</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>57.99</t>
@@ -1064,37 +960,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Celeste</t>
+          <t>Alexander</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Shields</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1520314</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>41004</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Herrings</t>
-        </is>
-      </c>
+          <t>Javitz</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>4.14.38</t>
-        </is>
-      </c>
+      <c r="H12" t="n">
+        <v>58</v>
+      </c>
+      <c r="I12" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1.57.93</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -1115,19 +1005,9 @@
           <t>Sanmartin Camba</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1718152</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>41431</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Herrings</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
         <v>59.47</v>
       </c>
@@ -1145,11 +1025,7 @@
           <t>2.14.75</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>4.18.63</t>
-        </is>
-      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>1.18.91</t>
@@ -1174,19 +1050,9 @@
           <t>Strasz</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1485250</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>41948</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>49.47</t>
@@ -1229,19 +1095,9 @@
           <t>Stojsavljevic</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1490856</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>41553</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>48.50</t>
@@ -1263,11 +1119,7 @@
           <t>1.55.09</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>3.42.38</t>
-        </is>
-      </c>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>57.47</t>
@@ -1292,19 +1144,9 @@
           <t>Sharma</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1596070</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>41246</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
@@ -1347,19 +1189,9 @@
           <t>O'Neill</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1510812</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="n">
-        <v>40982</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
@@ -1402,19 +1234,9 @@
           <t>Pelembe Habib</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1502644</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>40567</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -1424,11 +1246,7 @@
           <t>1.48.03</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>3.36.22</t>
-        </is>
-      </c>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
@@ -1466,23 +1284,13 @@
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" s="2" t="n">
-        <v>40437</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
@@ -1500,11 +1308,7 @@
           <t>2.31.25</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
@@ -1521,23 +1325,13 @@
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" s="2" t="n">
-        <v>40295</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
@@ -1555,11 +1349,7 @@
           <t>2.14.06</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
@@ -1576,23 +1366,13 @@
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" s="2" t="n">
-        <v>40809</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
@@ -1610,11 +1390,7 @@
           <t>2.15.75</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
@@ -1631,23 +1407,13 @@
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" s="2" t="n">
-        <v>39091</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Seals</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
@@ -1665,11 +1431,7 @@
           <t>2.14.47</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
@@ -1685,19 +1447,9 @@
           <t>Sharma</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1596067</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="n">
-        <v>40336</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Piranhas</t>
-        </is>
-      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1736,19 +1488,9 @@
           <t>Liebig-Koltai</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1473789</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="n">
-        <v>40296</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Piranhas</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1775,11 +1517,7 @@
           <t>1.50.38</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
@@ -1795,19 +1533,9 @@
           <t>Madden</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1611996</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="n">
-        <v>40193</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Piranhas</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1854,19 +1582,9 @@
           <t>Ujkaj</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1757344</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>39107</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Piranhas</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1876,32 +1594,16 @@
           <t>1.31.38</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
           <t>1.51.88</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
@@ -1917,19 +1619,9 @@
           <t>Romim</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1456822</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>40299</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Marlins</t>
-        </is>
-      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -1976,19 +1668,9 @@
           <t>Perkins</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>1499715</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>39936</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Marlins</t>
-        </is>
-      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -1998,11 +1680,7 @@
           <t>1.24.34</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>2.37.12</t>
-        </is>
-      </c>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
@@ -2039,19 +1717,9 @@
           <t>Davison</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1182267</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="n">
-        <v>39755</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Marlins</t>
-        </is>
-      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -2098,19 +1766,9 @@
           <t>Pollock</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1367549</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>39020</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Marlins</t>
-        </is>
-      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -2157,19 +1815,9 @@
           <t>Klos</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1438707</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>40125</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Marlins</t>
-        </is>
-      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -2179,11 +1827,7 @@
           <t>1.17.75</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>2.40.47</t>
-        </is>
-      </c>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
@@ -2220,19 +1864,9 @@
           <t>Savvanidis</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1256761</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>39472</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Marlins</t>
-        </is>
-      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -2259,11 +1893,7 @@
           <t>1.33.31</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
@@ -2279,19 +1909,9 @@
           <t>Koo</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1413299</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="n">
-        <v>39464</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Marlins</t>
-        </is>
-      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>

</xml_diff>

<commit_message>
fix - Added rest of information (dob, etc.) that was missing in extras table.
</commit_message>
<xml_diff>
--- a/extras.xlsx
+++ b/extras.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,9 +540,19 @@
           <t>Filmon</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1490851</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>41810</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Dolphins</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>1.11.50</t>
@@ -585,9 +599,19 @@
           <t>Myronov</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1673595</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>41951</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dolphins</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>55.09</t>
@@ -634,9 +658,19 @@
           <t>Smith</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1739168</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>41836</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Dolphins</t>
+        </is>
+      </c>
       <c r="F4" t="n">
         <v>58.25</v>
       </c>
@@ -677,9 +711,19 @@
           <t>Clarke</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1765402</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>42086</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Dolphins</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>54.91</v>
@@ -714,9 +758,19 @@
           <t>Peksa</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1648221</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>41211</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Dolphins</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>1.12.25</t>
@@ -755,9 +809,19 @@
           <t>Bellenger</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1772739</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>41353</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dolphins</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>1.11.25</t>
@@ -796,9 +860,19 @@
           <t>Obiamiwe</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1595685</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>41570</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Dolphins</t>
+        </is>
+      </c>
       <c r="F8" t="n">
         <v>53.81</v>
       </c>
@@ -841,9 +915,19 @@
           <t>Pitzioris</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1653488</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>41584</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Dolphins</t>
+        </is>
+      </c>
       <c r="F9" t="n">
         <v>59.38</v>
       </c>
@@ -878,9 +962,19 @@
           <t>Leung</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1684191</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>41946</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Herrings</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>59.91</t>
@@ -927,9 +1021,19 @@
           <t>O'Neill</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1592376</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>41919</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Herrings</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>57.99</t>
@@ -968,9 +1072,19 @@
           <t>Javitz</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1774121</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>42036</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Herrings</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
@@ -1005,9 +1119,19 @@
           <t>Sanmartin Camba</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1718152</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>41431</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Herrings</t>
+        </is>
+      </c>
       <c r="F13" t="n">
         <v>59.47</v>
       </c>
@@ -1050,9 +1174,19 @@
           <t>Strasz</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1485250</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>41948</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>49.47</t>
@@ -1095,9 +1229,19 @@
           <t>Stojsavljevic</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1490856</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>41553</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>48.50</t>
@@ -1144,9 +1288,19 @@
           <t>Sharma</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1596070</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>41246</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
@@ -1189,9 +1343,19 @@
           <t>O'Neill</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1510812</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>40982</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
@@ -1234,9 +1398,19 @@
           <t>Pelembe Habib</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1502644</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>40567</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -1284,8 +1458,14 @@
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="D19" s="2" t="n">
+        <v>40437</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -1325,8 +1505,14 @@
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="D20" s="2" t="n">
+        <v>40295</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -1366,8 +1552,14 @@
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="D21" s="2" t="n">
+        <v>40809</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -1407,8 +1599,14 @@
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="D22" s="2" t="n">
+        <v>39091</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -1447,9 +1645,19 @@
           <t>Sharma</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1596067</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>40336</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Piranhas</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1488,9 +1696,19 @@
           <t>Liebig-Koltai</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1473789</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>40296</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Piranhas</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1533,9 +1751,19 @@
           <t>Madden</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1611996</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>40193</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Piranhas</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1582,9 +1810,19 @@
           <t>Ujkaj</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1757344</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>39107</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Piranhas</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1619,9 +1857,19 @@
           <t>Romim</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1456822</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>40299</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Marlins</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -1668,9 +1916,19 @@
           <t>Perkins</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1499715</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>39936</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Marlins</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -1717,9 +1975,19 @@
           <t>Davison</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1182267</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>39755</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Marlins</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -1766,9 +2034,19 @@
           <t>Pollock</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1367549</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>39020</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Marlins</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -1815,9 +2093,19 @@
           <t>Klos</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1438707</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>40125</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Marlins</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -1864,9 +2152,19 @@
           <t>Savvanidis</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1256761</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>39472</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Marlins</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -1909,9 +2207,19 @@
           <t>Koo</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1413299</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>39464</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Marlins</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>

</xml_diff>